<commit_message>
agrega img ppal a 1er pag man
</commit_message>
<xml_diff>
--- a/bom/deTmpBasPdoffBor/deTmpBasPdoffBor.xlsx
+++ b/bom/deTmpBasPdoffBor/deTmpBasPdoffBor.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
   <si>
     <t>Description</t>
   </si>
@@ -25,9 +25,6 @@
     <t>C3</t>
   </si>
   <si>
-    <t>JP1</t>
-  </si>
-  <si>
     <t>K1</t>
   </si>
   <si>
@@ -37,9 +34,6 @@
     <t>1N4148 SMD</t>
   </si>
   <si>
-    <t>Cgrid Header 9x1</t>
-  </si>
-  <si>
     <t>N x100</t>
   </si>
   <si>
@@ -58,9 +52,6 @@
     <t>DL4148</t>
   </si>
   <si>
-    <t>TP1X40</t>
-  </si>
-  <si>
     <t>N x40</t>
   </si>
   <si>
@@ -70,9 +61,6 @@
     <t>VR085-10K</t>
   </si>
   <si>
-    <t>Total Materiales 1 unidad:</t>
-  </si>
-  <si>
     <t>Costo * N [US$]</t>
   </si>
   <si>
@@ -109,9 +97,6 @@
     <t>Zener 5.6V</t>
   </si>
   <si>
-    <t>D1, D2</t>
-  </si>
-  <si>
     <t>R5, R8</t>
   </si>
   <si>
@@ -122,6 +107,21 @@
   </si>
   <si>
     <t>D3</t>
+  </si>
+  <si>
+    <t>D1, D2, D4</t>
+  </si>
+  <si>
+    <t>Cgrid 4x1</t>
+  </si>
+  <si>
+    <t>jumper</t>
+  </si>
+  <si>
+    <t>bornera 3x1</t>
+  </si>
+  <si>
+    <t>bornera 2x1</t>
   </si>
 </sst>
 </file>
@@ -177,7 +177,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -187,12 +187,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -208,7 +202,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -235,13 +229,28 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -256,7 +265,7 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -265,13 +274,28 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -283,7 +307,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -298,7 +322,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -313,77 +337,12 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -391,30 +350,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -426,56 +400,29 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -772,7 +719,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="27" style="1" customWidth="1"/>
@@ -793,358 +740,336 @@
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="4" t="s">
+      <c r="I1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I1" s="7" t="s">
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="9">
+        <v>3</v>
+      </c>
+      <c r="D2" s="10">
+        <f t="shared" ref="D2:D10" si="0">C2*40</f>
+        <v>120</v>
+      </c>
+      <c r="E2" s="10">
+        <f t="shared" ref="E2:E10" si="1">100*C2</f>
+        <v>300</v>
+      </c>
+      <c r="F2" s="10">
+        <f t="shared" ref="F2:F10" si="2">D2*5</f>
+        <v>600</v>
+      </c>
+      <c r="G2" s="8">
+        <v>2.01E-2</v>
+      </c>
+      <c r="H2" s="8"/>
+      <c r="I2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J2" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="31.5">
+      <c r="A3" s="12" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" s="10">
+      <c r="B3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="9">
         <v>2</v>
       </c>
-      <c r="D2" s="11">
-        <f t="shared" ref="D2:D10" si="0">C2*40</f>
-        <v>80</v>
-      </c>
-      <c r="E2" s="11">
-        <f t="shared" ref="E2:E10" si="1">100*C2</f>
-        <v>200</v>
-      </c>
-      <c r="F2" s="11">
-        <f t="shared" ref="F2:F10" si="2">D2*5</f>
-        <v>400</v>
-      </c>
-      <c r="G2" s="9">
-        <v>2.01E-2</v>
-      </c>
-      <c r="H2" s="9"/>
-      <c r="I2" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="31.5">
-      <c r="A3" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="10">
-        <v>2</v>
-      </c>
-      <c r="D3" s="11">
+      <c r="D3" s="10">
         <f t="shared" ref="D3" si="3">C3*40</f>
         <v>80</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="10">
         <f t="shared" ref="E3" si="4">100*C3</f>
         <v>200</v>
       </c>
-      <c r="F3" s="11">
+      <c r="F3" s="10">
         <f t="shared" ref="F3" si="5">D3*5</f>
         <v>400</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="8">
         <v>6.7799999999999996E-3</v>
       </c>
-      <c r="H3" s="9"/>
-      <c r="I3" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" s="12" t="s">
+      <c r="H3" s="8"/>
+      <c r="I3" s="11" t="s">
         <v>21</v>
       </c>
+      <c r="J3" s="11" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="4" spans="1:10" ht="31.5">
-      <c r="A4" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="10">
+      <c r="A4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="9">
         <v>1</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="10">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="10">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="10">
         <f t="shared" si="2"/>
         <v>200</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="8">
         <v>6.7799999999999996E-3</v>
       </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="J4" s="12" t="s">
-        <v>21</v>
+      <c r="H4" s="8"/>
+      <c r="I4" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="10">
+      <c r="A5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="9">
         <v>1</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="10">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="10">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="10">
         <f t="shared" si="2"/>
         <v>200</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="8">
         <v>0.1278</v>
       </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12" t="s">
-        <v>21</v>
+      <c r="H5" s="8"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="47.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="15">
         <v>1</v>
       </c>
-      <c r="D6" s="17">
+      <c r="D6" s="16">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="E6" s="17">
+      <c r="E6" s="16">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="F6" s="17">
+      <c r="F6" s="16">
         <f t="shared" si="2"/>
         <v>200</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="14">
         <v>0.11094</v>
       </c>
-      <c r="H6" s="15"/>
-      <c r="I6" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="J6" s="18" t="s">
-        <v>22</v>
+      <c r="H6" s="14"/>
+      <c r="I6" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="15" t="s">
+      <c r="A7" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="14"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="20">
-        <f>1/4</f>
-        <v>0.25</v>
-      </c>
-      <c r="D7" s="17">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="E7" s="17">
-        <f t="shared" si="1"/>
-        <v>25</v>
-      </c>
-      <c r="F7" s="17">
-        <f t="shared" si="2"/>
-        <v>50</v>
-      </c>
-      <c r="G7" s="15">
-        <v>0.1734</v>
-      </c>
-      <c r="H7" s="15"/>
-      <c r="I7" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="J7" s="18" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="16">
+      <c r="C8" s="15">
         <v>1</v>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="16">
         <f t="shared" ref="D8" si="6">C8*40</f>
         <v>40</v>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="16">
         <f t="shared" ref="E8" si="7">100*C8</f>
         <v>100</v>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="16">
         <f t="shared" ref="F8" si="8">D8*5</f>
         <v>200</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="14">
         <v>0.61739999999999995</v>
       </c>
-      <c r="H8" s="15"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18" t="s">
-        <v>22</v>
+      <c r="H8" s="14"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="16">
+      <c r="C9" s="15">
         <v>1</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="16">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="16">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="16">
         <f t="shared" si="2"/>
         <v>200</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="14">
         <v>0.61739999999999995</v>
       </c>
-      <c r="H9" s="15"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18" t="s">
-        <v>22</v>
+      <c r="H9" s="14"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="48" thickBot="1">
-      <c r="A10" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="23">
+      <c r="A10" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="22">
         <v>1</v>
       </c>
-      <c r="D10" s="24">
+      <c r="D10" s="23">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="23">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="F10" s="24">
+      <c r="F10" s="23">
         <f t="shared" si="2"/>
         <v>200</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="21">
         <v>0.1182</v>
       </c>
-      <c r="H10" s="22"/>
-      <c r="I10" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="25" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="16.5" thickBot="1">
-      <c r="A11" s="27" t="s">
+      <c r="H10" s="21"/>
+      <c r="I10" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="J10" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="26">
-        <f>SUM(H2:H10)</f>
-        <v>0</v>
-      </c>
-      <c r="I11" s="6"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
       <c r="J11" s="5"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
+      <c r="A12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="1">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <sortState ref="A2:J9">
     <sortCondition ref="J2:J9"/>
   </sortState>
-  <mergeCells count="1">
-    <mergeCell ref="A11:G11"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>